<commit_message>
changed directionality of outcome variables, then changed them back (want 5 year change, not just periodic value I think)
</commit_message>
<xml_diff>
--- a/outputs/edge_stats_90m_RAN.xlsx
+++ b/outputs/edge_stats_90m_RAN.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raenb\Documents\GitHub\madagascar\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{7D2EF854-2CF9-44A4-967D-BB5F671B6A55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C21B115-CEA5-45B7-8FA1-DE36514D5555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-1035" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="edge_stats_90m" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -64,7 +61,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -4615,102 +4612,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="frag_stats_90m"/>
-      <sheetName val="reorganized"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="1">
-          <cell r="B1" t="str">
-            <v>National intactness</v>
-          </cell>
-          <cell r="C1" t="str">
-            <v>CFM intactness</v>
-          </cell>
-          <cell r="D1" t="str">
-            <v>PA intactness</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2">
-            <v>2005</v>
-          </cell>
-          <cell r="B2">
-            <v>64.819693069607993</v>
-          </cell>
-          <cell r="C2">
-            <v>73.805743493025005</v>
-          </cell>
-          <cell r="D2">
-            <v>85.0030203062054</v>
-          </cell>
-          <cell r="E2">
-            <v>30.599860180381501</v>
-          </cell>
-          <cell r="F2">
-            <v>26.087972027436098</v>
-          </cell>
-          <cell r="G2">
-            <v>21.195315081477901</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>2010</v>
-          </cell>
-          <cell r="B3">
-            <v>62.8706550428412</v>
-          </cell>
-          <cell r="C3">
-            <v>71.890855151157595</v>
-          </cell>
-          <cell r="D3">
-            <v>84.299214687961097</v>
-          </cell>
-          <cell r="E3">
-            <v>30.676056084584001</v>
-          </cell>
-          <cell r="F3">
-            <v>26.758623442522801</v>
-          </cell>
-          <cell r="G3">
-            <v>21.5320632582816</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>2014</v>
-          </cell>
-          <cell r="B4">
-            <v>60.617154869126999</v>
-          </cell>
-          <cell r="C4">
-            <v>69.366493733258395</v>
-          </cell>
-          <cell r="D4">
-            <v>83.329914590523302</v>
-          </cell>
-          <cell r="E4">
-            <v>30.658451814519299</v>
-          </cell>
-          <cell r="F4">
-            <v>27.279249385404899</v>
-          </cell>
-          <cell r="G4">
-            <v>21.948736070542999</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -5007,11 +4908,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>

</xml_diff>